<commit_message>
Updated Frosthaven Quest Cards until 96
</commit_message>
<xml_diff>
--- a/Frosthaven/! Quest Cards Frosthaven.xlsx
+++ b/Frosthaven/! Quest Cards Frosthaven.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\projects\haven\haven_quest_cards\Frosthaven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED064EB6-DA15-4E7A-8393-199557B5DF7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4DF166-FD7E-4657-BBFA-588A58A976F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="14370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -5677,7 +5677,40 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF555A"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{18BF88B3-45F5-48D8-8680-2CDA5B9CB784}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{18BF88B3-45F5-48D8-8680-2CDA5B9CB784}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFF555A"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D1:D1048576</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished rework of Frosthaven Quest Card Fronts
</commit_message>
<xml_diff>
--- a/Frosthaven/! Quest Cards Frosthaven.xlsx
+++ b/Frosthaven/! Quest Cards Frosthaven.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\projects\haven\haven_quest_cards\Frosthaven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4DF166-FD7E-4657-BBFA-588A58A976F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF6B458-E871-4376-AE07-EDADB3222819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="14370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="339">
   <si>
     <t>Chapter</t>
   </si>
@@ -1068,6 +1068,18 @@
   </si>
   <si>
     <t>Random Scenario</t>
+  </si>
+  <si>
+    <t>Other (Calendar)</t>
+  </si>
+  <si>
+    <t>Other (Event)</t>
+  </si>
+  <si>
+    <t>Other (Retirement)</t>
+  </si>
+  <si>
+    <t>Other (Building)</t>
   </si>
 </sst>
 </file>
@@ -4983,7 +4995,7 @@
         <v>113</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C115" s="10" t="s">
         <v>103</v>
@@ -5013,7 +5025,7 @@
         <v>114</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C116" s="5" t="s">
         <v>105</v>
@@ -5039,7 +5051,7 @@
         <v>115</v>
       </c>
       <c r="B117" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C117" s="5" t="s">
         <v>106</v>
@@ -5065,7 +5077,7 @@
         <v>116</v>
       </c>
       <c r="B118" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C118" s="5" t="s">
         <v>107</v>
@@ -5091,7 +5103,7 @@
         <v>117</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C119" s="5" t="s">
         <v>104</v>
@@ -5117,7 +5129,7 @@
         <v>118</v>
       </c>
       <c r="B120" s="28" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C120" s="5" t="s">
         <v>108</v>
@@ -5143,7 +5155,7 @@
         <v>119</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C121" s="5" t="s">
         <v>109</v>
@@ -5172,7 +5184,7 @@
         <v>120</v>
       </c>
       <c r="B122" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C122" s="5" t="s">
         <v>190</v>
@@ -5198,7 +5210,7 @@
         <v>121</v>
       </c>
       <c r="B123" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C123" s="10" t="s">
         <v>250</v>
@@ -5228,7 +5240,7 @@
         <v>122</v>
       </c>
       <c r="B124" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C124" s="5" t="s">
         <v>110</v>
@@ -5254,7 +5266,7 @@
         <v>123</v>
       </c>
       <c r="B125" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C125" s="10" t="s">
         <v>226</v>
@@ -5284,7 +5296,7 @@
         <v>124</v>
       </c>
       <c r="B126" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C126" s="5" t="s">
         <v>205</v>
@@ -5310,7 +5322,7 @@
         <v>125</v>
       </c>
       <c r="B127" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C127" s="5" t="s">
         <v>236</v>
@@ -5336,7 +5348,7 @@
         <v>126</v>
       </c>
       <c r="B128" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C128" s="5" t="s">
         <v>111</v>
@@ -5362,7 +5374,7 @@
         <v>127</v>
       </c>
       <c r="B129" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C129" s="5" t="s">
         <v>181</v>
@@ -5388,7 +5400,7 @@
         <v>128</v>
       </c>
       <c r="B130" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C130" s="10" t="s">
         <v>112</v>
@@ -5418,7 +5430,7 @@
         <v>129</v>
       </c>
       <c r="B131" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C131" s="5" t="s">
         <v>113</v>
@@ -5444,7 +5456,7 @@
         <v>130</v>
       </c>
       <c r="B132" s="28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C132" s="5" t="s">
         <v>219</v>
@@ -5473,7 +5485,7 @@
         <v>131</v>
       </c>
       <c r="B133" s="28" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C133" s="5" t="s">
         <v>261</v>
@@ -5557,7 +5569,7 @@
         <v>134</v>
       </c>
       <c r="B136" s="28" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C136" s="10" t="s">
         <v>117</v>
@@ -5587,7 +5599,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="28" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C137" s="10" t="s">
         <v>118</v>
@@ -5617,7 +5629,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="28" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C138" s="10" t="s">
         <v>119</v>
@@ -5649,7 +5661,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="28" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C139" s="10" t="s">
         <v>120</v>

</xml_diff>